<commit_message>
created master company database structure
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,35 +1,144 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nishantyadav/Documents/Career-Intelligence-System/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A10F57A-AD7A-E64A-97C4-1994BD10C7B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="17120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Targets" sheetId="1" r:id="rId1"/>
+    <sheet name="Keywords" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Career URL</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Keyword</t>
+  </si>
+  <si>
+    <t>Northvolt</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>https://career.northvolt.com</t>
+  </si>
+  <si>
+    <t>Battery manufacturer</t>
+  </si>
+  <si>
+    <t>CATL</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>https://career.catl.com</t>
+  </si>
+  <si>
+    <t>Fraunhofer</t>
+  </si>
+  <si>
+    <t>Research Institute</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>https://jobs.fraunhofer.de</t>
+  </si>
+  <si>
+    <t>Research institute</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Electrochemistry</t>
+  </si>
+  <si>
+    <t>Materials</t>
+  </si>
+  <si>
+    <t>Energy Storage</t>
+  </si>
+  <si>
+    <t>Research Engineer</t>
+  </si>
+  <si>
+    <t>OpenAI</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>https://boards.greenhouse.io/</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -44,84 +153,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -409,66 +463,174 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Career URL</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P10" s="2"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P11" s="2"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P12" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="https://career.northvolt.com/" xr:uid="{5D529C82-EC28-6047-8B0A-6294D53E9D4A}"/>
+    <hyperlink ref="D3" r:id="rId2" display="https://career.catl.com/" xr:uid="{3381B1AD-096D-7940-B70A-113E38ACFA32}"/>
+    <hyperlink ref="D4" r:id="rId3" display="https://jobs.fraunhofer.de/" xr:uid="{F9186282-C658-1541-BD71-6088104D64A5}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{F14B2E13-60F4-DB45-948D-80FCDB7FF371}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Keyword</t>
-        </is>
-      </c>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>